<commit_message>
new calibration data loaded
</commit_message>
<xml_diff>
--- a/Dimming_and_Pixel_Calibration_Sheet.xlsx
+++ b/Dimming_and_Pixel_Calibration_Sheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Documents\berk\roombrightening\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9633CE15-9F45-4B13-935D-24A4E261E2AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D47BDE9-66AE-4338-9429-2CA4C374F003}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4545" yWindow="2025" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Calibration Sheet" sheetId="1" r:id="rId1"/>
@@ -225,7 +225,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -236,12 +236,18 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -545,7 +551,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:K29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -555,24 +561,30 @@
     <col min="6" max="7" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="4" t="s">
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="5"/>
-      <c r="G1" s="4" t="s">
+      <c r="F1" s="6"/>
+      <c r="G1" s="5" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J1">
+        <v>34</v>
+      </c>
+      <c r="K1">
+        <v>1.1000000000000001</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -594,8 +606,14 @@
       <c r="G2" s="1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J2">
+        <v>48</v>
+      </c>
+      <c r="K2">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>9</v>
       </c>
@@ -617,8 +635,14 @@
       <c r="G3" s="2">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J3" s="7">
+        <v>58</v>
+      </c>
+      <c r="K3" s="8">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>10</v>
       </c>
@@ -638,8 +662,14 @@
       <c r="G4" s="3">
         <v>19.53</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J4">
+        <v>67</v>
+      </c>
+      <c r="K4">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>11</v>
       </c>
@@ -659,8 +689,14 @@
       <c r="G5" s="2">
         <v>39.04</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J5">
+        <v>74</v>
+      </c>
+      <c r="K5">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>12</v>
       </c>
@@ -680,8 +716,14 @@
       <c r="G6" s="3">
         <v>58.2</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J6">
+        <v>81</v>
+      </c>
+      <c r="K6">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>13</v>
       </c>
@@ -701,8 +743,14 @@
       <c r="G7" s="2">
         <v>77.099999999999994</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J7">
+        <v>87</v>
+      </c>
+      <c r="K7">
+        <v>1.7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>14</v>
       </c>
@@ -722,8 +770,14 @@
       <c r="G8" s="3">
         <v>95.7</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J8">
+        <v>93</v>
+      </c>
+      <c r="K8">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>15</v>
       </c>
@@ -743,8 +797,14 @@
       <c r="G9" s="2">
         <v>113.98</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J9">
+        <v>99</v>
+      </c>
+      <c r="K9">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>16</v>
       </c>
@@ -764,8 +824,14 @@
       <c r="G10" s="3">
         <v>131.57</v>
       </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J10">
+        <v>104</v>
+      </c>
+      <c r="K10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>17</v>
       </c>
@@ -785,8 +851,14 @@
       <c r="G11" s="2">
         <v>149.26</v>
       </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J11">
+        <v>109</v>
+      </c>
+      <c r="K11">
+        <v>2.1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>18</v>
       </c>
@@ -806,8 +878,14 @@
       <c r="G12" s="3">
         <v>167.4</v>
       </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J12">
+        <v>114</v>
+      </c>
+      <c r="K12">
+        <v>2.2000000000000002</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -827,8 +905,14 @@
       <c r="G13" s="2">
         <v>184.56</v>
       </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J13">
+        <v>119</v>
+      </c>
+      <c r="K13">
+        <v>2.2999999999999998</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>20</v>
       </c>
@@ -848,8 +932,14 @@
       <c r="G14" s="3">
         <v>203</v>
       </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J14">
+        <v>123</v>
+      </c>
+      <c r="K14">
+        <v>2.4</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>21</v>
       </c>
@@ -869,8 +959,14 @@
       <c r="G15" s="2">
         <v>218</v>
       </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J15">
+        <v>127</v>
+      </c>
+      <c r="K15">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>22</v>
       </c>
@@ -890,8 +986,14 @@
       <c r="G16" s="3">
         <v>235</v>
       </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J16">
+        <v>131</v>
+      </c>
+      <c r="K16">
+        <v>2.6</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>23</v>
       </c>
@@ -911,8 +1013,14 @@
       <c r="G17" s="2">
         <v>251</v>
       </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J17">
+        <v>135</v>
+      </c>
+      <c r="K17">
+        <v>2.7</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>24</v>
       </c>
@@ -932,8 +1040,14 @@
       <c r="G18" s="3">
         <v>266</v>
       </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J18">
+        <v>139</v>
+      </c>
+      <c r="K18">
+        <v>2.8</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>25</v>
       </c>
@@ -953,8 +1067,14 @@
       <c r="G19" s="2">
         <v>282</v>
       </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J19">
+        <v>143</v>
+      </c>
+      <c r="K19">
+        <v>2.9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>26</v>
       </c>
@@ -974,8 +1094,14 @@
       <c r="G20" s="3">
         <v>297</v>
       </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J20">
+        <v>147</v>
+      </c>
+      <c r="K20">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>27</v>
       </c>
@@ -996,7 +1122,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
         <v>28</v>
       </c>
@@ -1017,7 +1143,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>29</v>
       </c>
@@ -1038,7 +1164,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
         <v>30</v>
       </c>
@@ -1059,7 +1185,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>31</v>
       </c>
@@ -1080,7 +1206,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
         <v>32</v>
       </c>
@@ -1101,7 +1227,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>33</v>
       </c>
@@ -1122,7 +1248,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
         <v>34</v>
       </c>
@@ -1143,8 +1269,8 @@
         <v>412</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="D29" s="6">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D29" s="4">
         <v>155.77000000000001</v>
       </c>
       <c r="F29">

</xml_diff>

<commit_message>
dmx caculation changed per setup
</commit_message>
<xml_diff>
--- a/Dimming_and_Pixel_Calibration_Sheet.xlsx
+++ b/Dimming_and_Pixel_Calibration_Sheet.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Documents\berk\roombrightening\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aksu\roombrightening\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D47BDE9-66AE-4338-9429-2CA4C374F003}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F26179F-ADC1-4384-BDCE-C93846E9313A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -239,16 +239,16 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -562,19 +562,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="5" t="s">
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="6"/>
-      <c r="G1" s="5" t="s">
+      <c r="F1" s="8"/>
+      <c r="G1" s="7" t="s">
         <v>3</v>
       </c>
       <c r="J1">
@@ -635,10 +635,10 @@
       <c r="G3" s="2">
         <v>0</v>
       </c>
-      <c r="J3" s="7">
+      <c r="J3" s="5">
         <v>58</v>
       </c>
-      <c r="K3" s="8">
+      <c r="K3" s="6">
         <v>1.3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
dimming updated and learning block taken back
</commit_message>
<xml_diff>
--- a/Dimming_and_Pixel_Calibration_Sheet.xlsx
+++ b/Dimming_and_Pixel_Calibration_Sheet.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aksu\roombrightening\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Documents\berk\roombrightening\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F26179F-ADC1-4384-BDCE-C93846E9313A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C85231C8-0F4A-45DB-A532-0910F7D5B8D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="47">
   <si>
     <t>dimming</t>
   </si>
@@ -130,6 +130,42 @@
   </si>
   <si>
     <t>%100</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0-5</t>
+  </si>
+  <si>
+    <t>0-8</t>
+  </si>
+  <si>
+    <t>0-12</t>
+  </si>
+  <si>
+    <t>0-21</t>
+  </si>
+  <si>
+    <t>0-32</t>
+  </si>
+  <si>
+    <t>0-48</t>
+  </si>
+  <si>
+    <t>0-68</t>
+  </si>
+  <si>
+    <t>0-142</t>
+  </si>
+  <si>
+    <t>0-204</t>
+  </si>
+  <si>
+    <t>1-174</t>
+  </si>
+  <si>
+    <t>1-41</t>
+  </si>
+  <si>
+    <t>2-114</t>
   </si>
 </sst>
 </file>
@@ -225,7 +261,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -249,6 +285,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -551,7 +588,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K29"/>
+  <dimension ref="A1:K42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -643,640 +680,923 @@
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" s="3">
-        <v>10</v>
-      </c>
-      <c r="C4" s="3">
-        <v>61</v>
-      </c>
-      <c r="D4" s="3">
-        <v>5.01</v>
-      </c>
-      <c r="E4" s="3">
-        <v>10</v>
-      </c>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3">
-        <v>19.53</v>
-      </c>
-      <c r="J4">
-        <v>67</v>
-      </c>
-      <c r="K4">
-        <v>1.4</v>
-      </c>
+      <c r="A4" s="2"/>
+      <c r="B4" s="2">
+        <v>0</v>
+      </c>
+      <c r="C4" s="2">
+        <v>2</v>
+      </c>
+      <c r="D4" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2">
+        <v>0.03</v>
+      </c>
+      <c r="J4" s="5"/>
+      <c r="K4" s="6"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
-        <v>11</v>
-      </c>
+      <c r="A5" s="2"/>
       <c r="B5" s="2">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="C5" s="2">
-        <v>123</v>
+        <v>18</v>
       </c>
       <c r="D5" s="2">
-        <v>10.33</v>
-      </c>
-      <c r="E5" s="2">
-        <v>20</v>
-      </c>
+        <v>0.05</v>
+      </c>
+      <c r="E5" s="2"/>
       <c r="F5" s="2"/>
       <c r="G5" s="2">
-        <v>39.04</v>
-      </c>
-      <c r="J5">
-        <v>74</v>
-      </c>
-      <c r="K5">
-        <v>1.5</v>
-      </c>
+        <v>0.05</v>
+      </c>
+      <c r="H5" t="s">
+        <v>35</v>
+      </c>
+      <c r="J5" s="5"/>
+      <c r="K5" s="6"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" s="3">
-        <v>30</v>
-      </c>
-      <c r="C6" s="3">
-        <v>184</v>
-      </c>
-      <c r="D6" s="3">
-        <v>15.37</v>
-      </c>
-      <c r="E6" s="3">
-        <v>31</v>
-      </c>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3">
-        <v>58.2</v>
-      </c>
-      <c r="J6">
-        <v>81</v>
-      </c>
-      <c r="K6">
-        <v>1.6</v>
-      </c>
+      <c r="A6" s="2"/>
+      <c r="B6" s="2">
+        <v>0</v>
+      </c>
+      <c r="C6" s="2">
+        <v>25</v>
+      </c>
+      <c r="D6" s="2">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="H6" t="s">
+        <v>36</v>
+      </c>
+      <c r="J6" s="5"/>
+      <c r="K6" s="6"/>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
-        <v>13</v>
-      </c>
+      <c r="A7" s="2"/>
       <c r="B7" s="2">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="C7" s="2">
-        <v>246</v>
+        <v>39</v>
       </c>
       <c r="D7" s="2">
-        <v>20.37</v>
-      </c>
-      <c r="E7" s="2">
-        <v>41</v>
-      </c>
+        <v>0.1</v>
+      </c>
+      <c r="E7" s="2"/>
       <c r="F7" s="2"/>
       <c r="G7" s="2">
-        <v>77.099999999999994</v>
-      </c>
-      <c r="J7">
-        <v>87</v>
-      </c>
-      <c r="K7">
-        <v>1.7</v>
-      </c>
+        <v>0.1</v>
+      </c>
+      <c r="H7" t="s">
+        <v>37</v>
+      </c>
+      <c r="J7" s="5"/>
+      <c r="K7" s="6"/>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B8" s="3">
-        <v>51</v>
-      </c>
-      <c r="C8" s="3">
-        <v>51</v>
-      </c>
-      <c r="D8" s="3">
-        <v>25.4</v>
-      </c>
-      <c r="E8" s="3">
-        <v>51</v>
-      </c>
-      <c r="F8" s="3"/>
-      <c r="G8" s="3">
-        <v>95.7</v>
-      </c>
-      <c r="J8">
-        <v>93</v>
-      </c>
-      <c r="K8">
-        <v>1.8</v>
-      </c>
+      <c r="A8" s="2"/>
+      <c r="B8" s="2">
+        <v>0</v>
+      </c>
+      <c r="C8" s="2">
+        <v>66</v>
+      </c>
+      <c r="D8" s="2">
+        <v>0.15</v>
+      </c>
+      <c r="E8" s="2"/>
+      <c r="F8" s="2"/>
+      <c r="G8" s="2">
+        <v>0.15</v>
+      </c>
+      <c r="H8" t="s">
+        <v>38</v>
+      </c>
+      <c r="J8" s="5"/>
+      <c r="K8" s="6"/>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
-        <v>15</v>
-      </c>
+      <c r="A9" s="2"/>
       <c r="B9" s="2">
-        <v>61</v>
+        <v>0</v>
       </c>
       <c r="C9" s="2">
-        <v>112</v>
+        <v>94</v>
       </c>
       <c r="D9" s="2">
-        <v>30.33</v>
-      </c>
-      <c r="E9" s="2">
-        <v>61</v>
-      </c>
+        <v>0.22</v>
+      </c>
+      <c r="E9" s="2"/>
       <c r="F9" s="2"/>
       <c r="G9" s="2">
-        <v>113.98</v>
-      </c>
-      <c r="J9">
-        <v>99</v>
-      </c>
-      <c r="K9">
-        <v>1.9</v>
-      </c>
+        <v>0.22</v>
+      </c>
+      <c r="H9" t="s">
+        <v>39</v>
+      </c>
+      <c r="J9" s="5"/>
+      <c r="K9" s="6"/>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B10" s="3">
-        <v>71</v>
-      </c>
-      <c r="C10" s="3">
-        <v>174</v>
-      </c>
-      <c r="D10" s="3">
-        <v>35.22</v>
-      </c>
-      <c r="E10" s="3">
-        <v>71</v>
-      </c>
-      <c r="F10" s="3"/>
-      <c r="G10" s="3">
-        <v>131.57</v>
-      </c>
-      <c r="J10">
-        <v>104</v>
-      </c>
-      <c r="K10">
-        <v>2</v>
-      </c>
+      <c r="A10" s="2"/>
+      <c r="B10" s="2">
+        <v>0</v>
+      </c>
+      <c r="C10" s="2">
+        <v>133</v>
+      </c>
+      <c r="D10" s="2">
+        <v>0.32</v>
+      </c>
+      <c r="E10" s="2"/>
+      <c r="F10" s="2"/>
+      <c r="G10" s="2">
+        <v>0.32</v>
+      </c>
+      <c r="H10" t="s">
+        <v>40</v>
+      </c>
+      <c r="J10" s="5"/>
+      <c r="K10" s="6"/>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
-        <v>17</v>
-      </c>
+      <c r="A11" s="2"/>
       <c r="B11" s="2">
-        <v>81</v>
+        <v>0</v>
       </c>
       <c r="C11" s="2">
-        <v>235</v>
+        <v>187</v>
       </c>
       <c r="D11" s="2">
-        <v>40.700000000000003</v>
-      </c>
-      <c r="E11" s="2">
-        <v>82</v>
-      </c>
+        <v>0.47</v>
+      </c>
+      <c r="E11" s="2"/>
       <c r="F11" s="2"/>
       <c r="G11" s="2">
-        <v>149.26</v>
-      </c>
-      <c r="J11">
-        <v>109</v>
-      </c>
-      <c r="K11">
-        <v>2.1</v>
-      </c>
+        <v>0.47</v>
+      </c>
+      <c r="H11" t="s">
+        <v>41</v>
+      </c>
+      <c r="J11" s="5"/>
+      <c r="K11" s="6"/>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A12" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="B12" s="3">
-        <v>92</v>
-      </c>
-      <c r="C12" s="3">
-        <v>41</v>
-      </c>
-      <c r="D12" s="3">
-        <v>44.85</v>
-      </c>
-      <c r="E12" s="3">
-        <v>92</v>
-      </c>
-      <c r="F12" s="3"/>
-      <c r="G12" s="3">
-        <v>167.4</v>
-      </c>
-      <c r="J12">
-        <v>114</v>
-      </c>
-      <c r="K12">
-        <v>2.2000000000000002</v>
-      </c>
+      <c r="A12" s="2"/>
+      <c r="B12" s="2">
+        <v>1</v>
+      </c>
+      <c r="C12" s="2">
+        <v>136</v>
+      </c>
+      <c r="D12" s="2">
+        <v>1</v>
+      </c>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2">
+        <v>1</v>
+      </c>
+      <c r="H12" t="s">
+        <v>42</v>
+      </c>
+      <c r="J12" s="5"/>
+      <c r="K12" s="6"/>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="A13" s="2"/>
       <c r="B13" s="2">
-        <v>102</v>
+        <v>2</v>
       </c>
       <c r="C13" s="2">
-        <v>102</v>
+        <v>60</v>
       </c>
       <c r="D13" s="2">
-        <v>49.75</v>
-      </c>
-      <c r="E13" s="2">
-        <v>102</v>
-      </c>
+        <v>1.48</v>
+      </c>
+      <c r="E13" s="2"/>
       <c r="F13" s="2"/>
       <c r="G13" s="2">
-        <v>184.56</v>
-      </c>
-      <c r="J13">
-        <v>119</v>
-      </c>
-      <c r="K13">
-        <v>2.2999999999999998</v>
-      </c>
+        <v>1.48</v>
+      </c>
+      <c r="H13" t="s">
+        <v>43</v>
+      </c>
+      <c r="J13" s="5"/>
+      <c r="K13" s="6"/>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B14" s="3">
-        <v>112</v>
-      </c>
-      <c r="C14" s="3">
-        <v>163</v>
-      </c>
-      <c r="D14" s="3">
-        <v>54.44</v>
-      </c>
-      <c r="E14" s="3">
-        <v>112</v>
-      </c>
-      <c r="F14" s="3"/>
-      <c r="G14" s="3">
-        <v>203</v>
-      </c>
-      <c r="J14">
-        <v>123</v>
-      </c>
-      <c r="K14">
-        <v>2.4</v>
-      </c>
+      <c r="A14" s="2"/>
+      <c r="B14" s="2">
+        <v>3</v>
+      </c>
+      <c r="C14" s="2">
+        <v>54</v>
+      </c>
+      <c r="D14" s="2">
+        <v>2.16</v>
+      </c>
+      <c r="E14" s="2"/>
+      <c r="F14" s="2"/>
+      <c r="G14" s="2">
+        <v>2.16</v>
+      </c>
+      <c r="H14" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="J14" s="5"/>
+      <c r="K14" s="6"/>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A15" s="2" t="s">
-        <v>21</v>
-      </c>
+      <c r="A15" s="2"/>
       <c r="B15" s="2">
-        <v>122</v>
+        <v>4</v>
       </c>
       <c r="C15" s="2">
-        <v>225</v>
+        <v>174</v>
       </c>
       <c r="D15" s="2">
-        <v>59.11</v>
-      </c>
-      <c r="E15" s="2">
-        <v>122</v>
-      </c>
+        <v>3.16</v>
+      </c>
+      <c r="E15" s="2"/>
       <c r="F15" s="2"/>
       <c r="G15" s="2">
+        <v>3.16</v>
+      </c>
+      <c r="H15" t="s">
+        <v>44</v>
+      </c>
+      <c r="J15" s="5"/>
+      <c r="K15" s="6"/>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A16" s="2"/>
+      <c r="B16" s="2">
+        <v>6</v>
+      </c>
+      <c r="C16" s="2">
+        <v>224</v>
+      </c>
+      <c r="D16" s="2">
+        <v>4.6399999999999997</v>
+      </c>
+      <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="2">
+        <v>4.6399999999999997</v>
+      </c>
+      <c r="H16" t="s">
+        <v>46</v>
+      </c>
+      <c r="J16" s="5"/>
+      <c r="K16" s="6"/>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B17" s="3">
+        <v>10</v>
+      </c>
+      <c r="C17" s="3">
+        <v>61</v>
+      </c>
+      <c r="D17" s="3">
+        <v>5.01</v>
+      </c>
+      <c r="E17" s="3">
+        <v>10</v>
+      </c>
+      <c r="F17" s="3"/>
+      <c r="G17" s="3">
+        <v>19.53</v>
+      </c>
+      <c r="J17">
+        <v>67</v>
+      </c>
+      <c r="K17">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B18" s="2">
+        <v>20</v>
+      </c>
+      <c r="C18" s="2">
+        <v>123</v>
+      </c>
+      <c r="D18" s="2">
+        <v>10.33</v>
+      </c>
+      <c r="E18" s="2">
+        <v>20</v>
+      </c>
+      <c r="F18" s="2"/>
+      <c r="G18" s="2">
+        <v>39.04</v>
+      </c>
+      <c r="J18">
+        <v>74</v>
+      </c>
+      <c r="K18">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B19" s="3">
+        <v>30</v>
+      </c>
+      <c r="C19" s="3">
+        <v>184</v>
+      </c>
+      <c r="D19" s="3">
+        <v>15.37</v>
+      </c>
+      <c r="E19" s="3">
+        <v>31</v>
+      </c>
+      <c r="F19" s="3"/>
+      <c r="G19" s="3">
+        <v>58.2</v>
+      </c>
+      <c r="J19">
+        <v>81</v>
+      </c>
+      <c r="K19">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B20" s="2">
+        <v>40</v>
+      </c>
+      <c r="C20" s="2">
+        <v>246</v>
+      </c>
+      <c r="D20" s="2">
+        <v>20.37</v>
+      </c>
+      <c r="E20" s="2">
+        <v>41</v>
+      </c>
+      <c r="F20" s="2"/>
+      <c r="G20" s="2">
+        <v>77.099999999999994</v>
+      </c>
+      <c r="J20">
+        <v>87</v>
+      </c>
+      <c r="K20">
+        <v>1.7</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B21" s="3">
+        <v>51</v>
+      </c>
+      <c r="C21" s="3">
+        <v>51</v>
+      </c>
+      <c r="D21" s="3">
+        <v>25.4</v>
+      </c>
+      <c r="E21" s="3">
+        <v>51</v>
+      </c>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3">
+        <v>95.7</v>
+      </c>
+      <c r="J21">
+        <v>93</v>
+      </c>
+      <c r="K21">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B22" s="2">
+        <v>61</v>
+      </c>
+      <c r="C22" s="2">
+        <v>112</v>
+      </c>
+      <c r="D22" s="2">
+        <v>30.33</v>
+      </c>
+      <c r="E22" s="2">
+        <v>61</v>
+      </c>
+      <c r="F22" s="2"/>
+      <c r="G22" s="2">
+        <v>113.98</v>
+      </c>
+      <c r="J22">
+        <v>99</v>
+      </c>
+      <c r="K22">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B23" s="3">
+        <v>71</v>
+      </c>
+      <c r="C23" s="3">
+        <v>174</v>
+      </c>
+      <c r="D23" s="3">
+        <v>35.22</v>
+      </c>
+      <c r="E23" s="3">
+        <v>71</v>
+      </c>
+      <c r="F23" s="3"/>
+      <c r="G23" s="3">
+        <v>131.57</v>
+      </c>
+      <c r="J23">
+        <v>104</v>
+      </c>
+      <c r="K23">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B24" s="2">
+        <v>81</v>
+      </c>
+      <c r="C24" s="2">
+        <v>235</v>
+      </c>
+      <c r="D24" s="2">
+        <v>40.700000000000003</v>
+      </c>
+      <c r="E24" s="2">
+        <v>82</v>
+      </c>
+      <c r="F24" s="2"/>
+      <c r="G24" s="2">
+        <v>149.26</v>
+      </c>
+      <c r="J24">
+        <v>109</v>
+      </c>
+      <c r="K24">
+        <v>2.1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B25" s="3">
+        <v>92</v>
+      </c>
+      <c r="C25" s="3">
+        <v>41</v>
+      </c>
+      <c r="D25" s="3">
+        <v>44.85</v>
+      </c>
+      <c r="E25" s="3">
+        <v>92</v>
+      </c>
+      <c r="F25" s="3"/>
+      <c r="G25" s="3">
+        <v>167.4</v>
+      </c>
+      <c r="J25">
+        <v>114</v>
+      </c>
+      <c r="K25">
+        <v>2.2000000000000002</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B26" s="2">
+        <v>102</v>
+      </c>
+      <c r="C26" s="2">
+        <v>102</v>
+      </c>
+      <c r="D26" s="2">
+        <v>49.75</v>
+      </c>
+      <c r="E26" s="2">
+        <v>102</v>
+      </c>
+      <c r="F26" s="2"/>
+      <c r="G26" s="2">
+        <v>184.56</v>
+      </c>
+      <c r="J26">
+        <v>119</v>
+      </c>
+      <c r="K26">
+        <v>2.2999999999999998</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A27" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B27" s="3">
+        <v>112</v>
+      </c>
+      <c r="C27" s="3">
+        <v>163</v>
+      </c>
+      <c r="D27" s="3">
+        <v>54.44</v>
+      </c>
+      <c r="E27" s="3">
+        <v>112</v>
+      </c>
+      <c r="F27" s="3"/>
+      <c r="G27" s="3">
+        <v>203</v>
+      </c>
+      <c r="J27">
+        <v>123</v>
+      </c>
+      <c r="K27">
+        <v>2.4</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B28" s="2">
+        <v>122</v>
+      </c>
+      <c r="C28" s="2">
+        <v>225</v>
+      </c>
+      <c r="D28" s="2">
+        <v>59.11</v>
+      </c>
+      <c r="E28" s="2">
+        <v>122</v>
+      </c>
+      <c r="F28" s="2"/>
+      <c r="G28" s="2">
         <v>218</v>
       </c>
-      <c r="J15">
+      <c r="J28">
         <v>127</v>
       </c>
-      <c r="K15">
+      <c r="K28">
         <v>2.5</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A16" s="3" t="s">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A29" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B16" s="3">
+      <c r="B29" s="3">
         <v>133</v>
       </c>
-      <c r="C16" s="3">
+      <c r="C29" s="3">
         <v>30</v>
       </c>
-      <c r="D16" s="3">
+      <c r="D29" s="3">
         <v>63.83</v>
       </c>
-      <c r="E16" s="3">
+      <c r="E29" s="3">
         <v>133</v>
       </c>
-      <c r="F16" s="3"/>
-      <c r="G16" s="3">
+      <c r="F29" s="3"/>
+      <c r="G29" s="3">
         <v>235</v>
       </c>
-      <c r="J16">
+      <c r="J29">
         <v>131</v>
       </c>
-      <c r="K16">
+      <c r="K29">
         <v>2.6</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A17" s="2" t="s">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A30" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B17" s="2">
+      <c r="B30" s="2">
         <v>143</v>
       </c>
-      <c r="C17" s="2">
+      <c r="C30" s="2">
         <v>92</v>
       </c>
-      <c r="D17" s="2">
+      <c r="D30" s="2">
         <v>68.760000000000005</v>
       </c>
-      <c r="E17" s="2">
+      <c r="E30" s="2">
         <v>143</v>
       </c>
-      <c r="F17" s="2"/>
-      <c r="G17" s="2">
+      <c r="F30" s="2"/>
+      <c r="G30" s="2">
         <v>251</v>
       </c>
-      <c r="J17">
+      <c r="J30">
         <v>135</v>
       </c>
-      <c r="K17">
+      <c r="K30">
         <v>2.7</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A18" s="3" t="s">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A31" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B18" s="3">
+      <c r="B31" s="3">
         <v>153</v>
       </c>
-      <c r="C18" s="3">
+      <c r="C31" s="3">
         <v>153</v>
       </c>
-      <c r="D18" s="3">
+      <c r="D31" s="3">
         <v>73.459999999999994</v>
       </c>
-      <c r="E18" s="3">
+      <c r="E31" s="3">
         <v>153</v>
       </c>
-      <c r="F18" s="3"/>
-      <c r="G18" s="3">
+      <c r="F31" s="3"/>
+      <c r="G31" s="3">
         <v>266</v>
       </c>
-      <c r="J18">
+      <c r="J31">
         <v>139</v>
       </c>
-      <c r="K18">
+      <c r="K31">
         <v>2.8</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A19" s="2" t="s">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A32" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B19" s="2">
+      <c r="B32" s="2">
         <v>163</v>
       </c>
-      <c r="C19" s="2">
+      <c r="C32" s="2">
         <v>214</v>
       </c>
-      <c r="D19" s="2">
+      <c r="D32" s="2">
         <v>77.75</v>
       </c>
-      <c r="E19" s="2">
+      <c r="E32" s="2">
         <v>163</v>
       </c>
-      <c r="F19" s="2"/>
-      <c r="G19" s="2">
+      <c r="F32" s="2"/>
+      <c r="G32" s="2">
         <v>282</v>
       </c>
-      <c r="J19">
+      <c r="J32">
         <v>143</v>
       </c>
-      <c r="K19">
+      <c r="K32">
         <v>2.9</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A20" s="3" t="s">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A33" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B20" s="3">
+      <c r="B33" s="3">
         <v>174</v>
       </c>
-      <c r="C20" s="3">
+      <c r="C33" s="3">
         <v>20</v>
       </c>
-      <c r="D20" s="3">
+      <c r="D33" s="3">
         <v>82.27</v>
       </c>
-      <c r="E20" s="3">
+      <c r="E33" s="3">
         <v>173</v>
       </c>
-      <c r="F20" s="3"/>
-      <c r="G20" s="3">
+      <c r="F33" s="3"/>
+      <c r="G33" s="3">
         <v>297</v>
       </c>
-      <c r="J20">
+      <c r="J33">
         <v>147</v>
       </c>
-      <c r="K20">
+      <c r="K33">
         <v>3</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A21" s="2" t="s">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A34" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B21" s="2">
+      <c r="B34" s="2">
         <v>184</v>
       </c>
-      <c r="C21" s="2">
+      <c r="C34" s="2">
         <v>81</v>
       </c>
-      <c r="D21" s="2">
+      <c r="D34" s="2">
         <v>86.65</v>
       </c>
-      <c r="E21" s="2">
+      <c r="E34" s="2">
         <v>184</v>
       </c>
-      <c r="F21" s="2"/>
-      <c r="G21" s="2">
+      <c r="F34" s="2"/>
+      <c r="G34" s="2">
         <v>312</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A22" s="3" t="s">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A35" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B22" s="3">
+      <c r="B35" s="3">
         <v>194</v>
       </c>
-      <c r="C22" s="3">
+      <c r="C35" s="3">
         <v>143</v>
       </c>
-      <c r="D22" s="3">
+      <c r="D35" s="3">
         <v>90.92</v>
       </c>
-      <c r="E22" s="3">
+      <c r="E35" s="3">
         <v>194</v>
       </c>
-      <c r="F22" s="3"/>
-      <c r="G22" s="3">
+      <c r="F35" s="3"/>
+      <c r="G35" s="3">
         <v>326</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A23" s="2" t="s">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A36" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B23" s="2">
+      <c r="B36" s="2">
         <v>204</v>
       </c>
-      <c r="C23" s="2">
+      <c r="C36" s="2">
         <v>204</v>
       </c>
-      <c r="D23" s="2">
+      <c r="D36" s="2">
         <v>95.14</v>
       </c>
-      <c r="E23" s="2">
+      <c r="E36" s="2">
         <v>204</v>
       </c>
-      <c r="F23" s="2"/>
-      <c r="G23" s="2">
+      <c r="F36" s="2"/>
+      <c r="G36" s="2">
         <v>341</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A24" s="3" t="s">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A37" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B24" s="3">
+      <c r="B37" s="3">
         <v>215</v>
       </c>
-      <c r="C24" s="3">
+      <c r="C37" s="3">
         <v>9</v>
       </c>
-      <c r="D24" s="3">
+      <c r="D37" s="3">
         <v>99.74</v>
       </c>
-      <c r="E24" s="3">
+      <c r="E37" s="3">
         <v>214</v>
       </c>
-      <c r="F24" s="3"/>
-      <c r="G24" s="3">
+      <c r="F37" s="3"/>
+      <c r="G37" s="3">
         <v>355</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A25" s="2" t="s">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A38" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B25" s="2">
+      <c r="B38" s="2">
         <v>225</v>
       </c>
-      <c r="C25" s="2">
+      <c r="C38" s="2">
         <v>71</v>
       </c>
-      <c r="D25" s="2">
+      <c r="D38" s="2">
         <v>103.76</v>
       </c>
-      <c r="E25" s="2">
+      <c r="E38" s="2">
         <v>224</v>
       </c>
-      <c r="F25" s="2"/>
-      <c r="G25" s="2">
+      <c r="F38" s="2"/>
+      <c r="G38" s="2">
         <v>369</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A26" s="3" t="s">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A39" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="B26" s="3">
+      <c r="B39" s="3">
         <v>235</v>
       </c>
-      <c r="C26" s="3">
+      <c r="C39" s="3">
         <v>132</v>
       </c>
-      <c r="D26" s="3">
+      <c r="D39" s="3">
         <v>107.94</v>
       </c>
-      <c r="E26" s="3">
+      <c r="E39" s="3">
         <v>235</v>
       </c>
-      <c r="F26" s="3"/>
-      <c r="G26" s="3">
+      <c r="F39" s="3"/>
+      <c r="G39" s="3">
         <v>382</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A27" s="2" t="s">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A40" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B27" s="2">
+      <c r="B40" s="2">
         <v>245</v>
       </c>
-      <c r="C27" s="2">
+      <c r="C40" s="2">
         <v>194</v>
       </c>
-      <c r="D27" s="2">
+      <c r="D40" s="2">
         <v>111.91</v>
       </c>
-      <c r="E27" s="2">
+      <c r="E40" s="2">
         <v>245</v>
       </c>
-      <c r="F27" s="2"/>
-      <c r="G27" s="2">
+      <c r="F40" s="2"/>
+      <c r="G40" s="2">
         <v>395</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A28" s="3" t="s">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A41" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="B28" s="3">
+      <c r="B41" s="3">
         <v>255</v>
       </c>
-      <c r="C28" s="3">
+      <c r="C41" s="3">
         <v>255</v>
       </c>
-      <c r="D28" s="3">
+      <c r="D41" s="3">
         <v>116.4</v>
       </c>
-      <c r="E28" s="3">
+      <c r="E41" s="3">
         <v>255</v>
       </c>
-      <c r="F28" s="3"/>
-      <c r="G28" s="3">
+      <c r="F41" s="3"/>
+      <c r="G41" s="3">
         <v>412</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="D29" s="4">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D42" s="4">
         <v>155.77000000000001</v>
       </c>
-      <c r="F29">
+      <c r="F42">
         <v>914</v>
       </c>
-      <c r="G29">
+      <c r="G42">
         <v>415</v>
       </c>
     </row>
@@ -1288,5 +1608,6 @@
     <mergeCell ref="D1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>